<commit_message>
Update Yandex Interview Kit (38/71)
</commit_message>
<xml_diff>
--- a/interview-materials/Yandex Interview Kit.xlsx
+++ b/interview-materials/Yandex Interview Kit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\personal\java-interview-coding\interview-materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A41FE24-02E3-4A40-85B0-497B8EF95C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44F9384D-FC17-40F8-A80A-AF34DF5EC27B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -670,7 +670,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="17">
-        <v>30</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.25">
@@ -803,7 +803,7 @@
       <c r="A11" s="5">
         <v>21</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="16" t="s">
         <v>44</v>
       </c>
       <c r="C11" s="7">
@@ -845,7 +845,7 @@
       <c r="A14" s="1">
         <v>232</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="16" t="s">
         <v>41</v>
       </c>
       <c r="C14" s="3">
@@ -859,7 +859,7 @@
       <c r="A15" s="5">
         <v>387</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="16" t="s">
         <v>74</v>
       </c>
       <c r="C15" s="7">
@@ -915,7 +915,7 @@
       <c r="A19" s="5">
         <v>392</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="16" t="s">
         <v>54</v>
       </c>
       <c r="C19" s="7">
@@ -999,7 +999,7 @@
       <c r="A25" s="1">
         <v>88</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="16" t="s">
         <v>43</v>
       </c>
       <c r="C25" s="3">
@@ -1335,7 +1335,7 @@
       <c r="A49" s="5">
         <v>438</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C49" s="7">
@@ -1377,7 +1377,7 @@
       <c r="A52" s="5">
         <v>56</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C52" s="7">
@@ -1461,7 +1461,7 @@
       <c r="A58" s="5">
         <v>2</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C58" s="7">

</xml_diff>